<commit_message>
Agregar registro de uso de IA de Johan Gallardo en Fase 1
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias grupales/Plantilla_Registro_Uso_IA_Capstone.xlsx
+++ b/FASE 1/Evidencias grupales/Plantilla_Registro_Uso_IA_Capstone.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
   <si>
     <t>Fase</t>
   </si>
@@ -90,6 +90,36 @@
   </si>
   <si>
     <t>El contenido generado fue revisado y adaptado íntegramente por el equipo antes de incorporarlo al entregable.</t>
+  </si>
+  <si>
+    <t>Johan Gallardo</t>
+  </si>
+  <si>
+    <t>Claude Code (Anthropic)</t>
+  </si>
+  <si>
+    <t>Claude Opus 5.5</t>
+  </si>
+  <si>
+    <t>Desarrollar el backend de AgroSense, integrar el frontend (mockup) con datos reales, conectar las lecturas del dispositivo ESP32 vía Firebase y desplegar la plataforma en producción.</t>
+  </si>
+  <si>
+    <t>"Clona el repositorio AgroSense; el frontend está en mockup, le falta login y no tiene backend. Necesito construir el backend completo con PostgreSQL, integrar Firebase para recibir las lecturas del dispositivo, ajustar el front a lo que realmente tenemos y desplegarlo en un VPS de Hostinger".</t>
+  </si>
+  <si>
+    <t>API REST en .NET 10 con PostgreSQL y autenticación (login), servicio que lee Firebase Realtime Database cada 10 s, simulador del ESP32, 20 pruebas automatizadas, frontend React integrado y despliegue con Docker y HTTPS en agrosense.tech.</t>
+  </si>
+  <si>
+    <t>Definición de las decisiones técnicas (PostgreSQL, .NET 10), creación y configuración del proyecto Firebase y sus reglas, contratación y configuración del VPS y del dominio, y revisión del código antes de integrarlo (pull request #1).</t>
+  </si>
+  <si>
+    <t>Ejecución de las pruebas automatizadas, pruebas de extremo a extremo con el simulador del ESP32 y verificación del sitio y la API funcionando en producción.</t>
+  </si>
+  <si>
+    <t>Permitió construir y desplegar en una jornada el backend y la integración que el proyecto no tenía; mayor calidad por las pruebas automatizadas y un despliegue reproducible.</t>
+  </si>
+  <si>
+    <t>El código generado fue revisado e integrado por el integrante. Las credenciales y claves se mantuvieron fuera del repositorio.</t>
   </si>
 </sst>
 </file>
@@ -534,6 +564,44 @@
       </c>
       <c r="L2" s="2" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="3">
+        <v>46297.0</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>